<commit_message>
769 NE 74th Rev 2: anchors 9 boxes (3 rows @ 12in)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp3FWjZDHZyKTZa15Tj1vA
</commit_message>
<xml_diff>
--- a/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev2.xlsx
+++ b/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev2.xlsx
@@ -748,11 +748,11 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2 term bar rows + counterflashing @ 12" o.c. (~580)</t>
+          <t>3 rows @ 12" o.c.: 2 term bar + counterflashing (787 +10% = 866)</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
769 NE 74th Rev 2: add brushes, bits, rollers, mops
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp3FWjZDHZyKTZa15Tj1vA
</commit_message>
<xml_diff>
--- a/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev2.xlsx
+++ b/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev2.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -953,36 +953,221 @@
       </c>
       <c r="H15" s="3" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Brushes 4"</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Brush 4</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Adhesive/primer cut-in</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="G16" s="4">
+        <f>D16*F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Shop price list 6/26/26</t>
+        </is>
+      </c>
+    </row>
     <row r="17">
-      <c r="F17" s="5" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Drill bits (masonry)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Drill bits</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>For 866 masonry anchors</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="G17" s="4">
+        <f>D17*F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Shop price list 6/26/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Roller frames 9" HD</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>C&amp;R 9" heavy duty roller frame #RF9HDN1</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Bonding adhesive application</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="G18" s="4">
+        <f>D18*F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Gulfeagle inv 2/5/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Roller covers 9" 3/4" nap</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>C&amp;R 9" roller cover 3/4" nap #RC9-3/4</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Bonding adhesive application</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G19" s="4">
+        <f>D19*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Gulfeagle inv 2/5/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Mops</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Mop</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="G20" s="4">
+        <f>D20*F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Shop price list 6/26/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Material subtotal</t>
         </is>
       </c>
-      <c r="G17" s="6">
-        <f>SUM(G4:G15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="F18" s="5" t="inlineStr">
+      <c r="G22" s="6">
+        <f>SUM(G4:G20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Sales tax 7%</t>
         </is>
       </c>
-      <c r="G18" s="6">
-        <f>ROUND(G17*0.07,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="F19" s="5" t="inlineStr">
+      <c r="G23" s="6">
+        <f>ROUND(G22*0.07,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>TOTAL MATERIAL</t>
         </is>
       </c>
-      <c r="G19" s="6">
-        <f>G17+G18</f>
+      <c r="G24" s="6">
+        <f>G22+G23</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
769 NE 74th Rev 2: revised tapered ISO $12,929
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp3FWjZDHZyKTZa15Tj1vA
</commit_message>
<xml_diff>
--- a/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev2.xlsx
+++ b/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev2.xlsx
@@ -669,7 +669,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>GAF EnergyGuard tapered ISO — Gulfeagle 25-1454-V3</t>
+          <t>GAF EnergyGuard tapered ISO — Gulfeagle revised quote</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>11971</v>
+        <v>12929</v>
       </c>
       <c r="G8" s="4">
         <f>D8*F8</f>
@@ -694,7 +694,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Quote expired 7/30/2025 — requote</t>
+          <t>Revised Gulfeagle quote per Marc 10/20/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
769 NE 74th Rev 2: VTR pipe boots from P-2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp3FWjZDHZyKTZa15Tj1vA
</commit_message>
<xml_diff>
--- a/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev2.xlsx
+++ b/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev2.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -956,21 +956,21 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Brushes 4"</t>
+          <t>Pipe boots 1"-2"</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Brush 4</t>
+          <t>GAF TPO split pipe boot 1"-2" white #85G1920</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Adhesive/primer cut-in</t>
+          <t>2" VTRs per P-2: master bath (2), Bath 1, Bath 2, Bath 3</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>1.47</v>
+        <v>38.51</v>
       </c>
       <c r="G16" s="4">
         <f>D16*F16</f>
@@ -986,24 +986,24 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Shop price list 6/26/26</t>
+          <t>Gulfeagle inv 2/4/26</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Drill bits (masonry)</t>
+          <t>Brushes 4"</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Drill bits</t>
+          <t>Brush 4</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>For 866 masonry anchors</t>
+          <t>Adhesive/primer cut-in</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>2.64</v>
+        <v>1.47</v>
       </c>
       <c r="G17" s="4">
         <f>D17*F17</f>
@@ -1030,21 +1030,21 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Roller frames 9" HD</t>
+          <t>Drill bits (masonry)</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>C&amp;R 9" heavy duty roller frame #RF9HDN1</t>
+          <t>Drill bits</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Bonding adhesive application</t>
+          <t>For 866 masonry anchors</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>2.7</v>
+        <v>2.64</v>
       </c>
       <c r="G18" s="4">
         <f>D18*F18</f>
@@ -1060,19 +1060,19 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Gulfeagle inv 2/5/26</t>
+          <t>Shop price list 6/26/26</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Roller covers 9" 3/4" nap</t>
+          <t>Roller frames 9" HD</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>C&amp;R 9" roller cover 3/4" nap #RC9-3/4</t>
+          <t>C&amp;R 9" heavy duty roller frame #RF9HDN1</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>1.65</v>
+        <v>2.7</v>
       </c>
       <c r="G19" s="4">
         <f>D19*F19</f>
@@ -1104,21 +1104,21 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Mops</t>
+          <t>Roller covers 9" 3/4" nap</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Mop</t>
+          <t>C&amp;R 9" roller cover 3/4" nap #RC9-3/4</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Job</t>
+          <t>Bonding adhesive application</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>7.15</v>
+        <v>1.65</v>
       </c>
       <c r="G20" s="4">
         <f>D20*F20</f>
@@ -1134,40 +1134,77 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
+          <t>Gulfeagle inv 2/5/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Mops</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Mop</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="G21" s="4">
+        <f>D21*F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
           <t>Shop price list 6/26/26</t>
         </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Material subtotal</t>
-        </is>
-      </c>
-      <c r="G22" s="6">
-        <f>SUM(G4:G20)</f>
-        <v/>
       </c>
     </row>
     <row r="23">
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Sales tax 7%</t>
+          <t>Material subtotal</t>
         </is>
       </c>
       <c r="G23" s="6">
-        <f>ROUND(G22*0.07,2)</f>
+        <f>SUM(G4:G21)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="F24" s="5" t="inlineStr">
         <is>
+          <t>Sales tax 7%</t>
+        </is>
+      </c>
+      <c r="G24" s="6">
+        <f>ROUND(G23*0.07,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="F25" s="5" t="inlineStr">
+        <is>
           <t>TOTAL MATERIAL</t>
         </is>
       </c>
-      <c r="G24" s="6">
-        <f>G22+G23</f>
+      <c r="G25" s="6">
+        <f>G23+G24</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
769 NE 74th Rev 2: TPO scuppers + 3in boot from Gulfeagle quote; save quote to reference
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp3FWjZDHZyKTZa15Tj1vA
</commit_message>
<xml_diff>
--- a/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev2.xlsx
+++ b/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev2.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -993,21 +993,21 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Brushes 4"</t>
+          <t>Pipe boot 3"-5" (laundry 3" VTR)</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Brush 4</t>
+          <t>GAF TPO split pipe boot 3"-5" white #85G2920</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Adhesive/primer cut-in</t>
+          <t>3" VTR per P-2</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>1.47</v>
+        <v>45.45</v>
       </c>
       <c r="G17" s="4">
         <f>D17*F17</f>
@@ -1023,28 +1023,28 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Shop price list 6/26/26</t>
+          <t>Gulfeagle quote S002031839 12/12/24</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Drill bits (masonry)</t>
+          <t>TPO scuppers (4 primary + 4 overflow)</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Drill bits</t>
+          <t>GAF EverGuard TPO scupper 8x10x12 white #B5TB920</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>For 866 masonry anchors</t>
+          <t>10"x4" openings per P-3; 12" throat for 8" CMU + stucco</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>2.64</v>
+        <v>212.75</v>
       </c>
       <c r="G18" s="4">
         <f>D18*F18</f>
@@ -1060,28 +1060,28 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Shop price list 6/26/26</t>
+          <t>Gulfeagle quote S002031839 12/12/24 — reconfirm</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Roller frames 9" HD</t>
+          <t>Brushes 4"</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>C&amp;R 9" heavy duty roller frame #RF9HDN1</t>
+          <t>Brush 4</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Bonding adhesive application</t>
+          <t>Adhesive/primer cut-in</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>2.7</v>
+        <v>1.47</v>
       </c>
       <c r="G19" s="4">
         <f>D19*F19</f>
@@ -1097,28 +1097,28 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Gulfeagle inv 2/5/26</t>
+          <t>Shop price list 6/26/26</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Roller covers 9" 3/4" nap</t>
+          <t>Drill bits (masonry)</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>C&amp;R 9" roller cover 3/4" nap #RC9-3/4</t>
+          <t>Drill bits</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Bonding adhesive application</t>
+          <t>For 866 masonry anchors</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>1.65</v>
+        <v>2.64</v>
       </c>
       <c r="G20" s="4">
         <f>D20*F20</f>
@@ -1134,28 +1134,28 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Gulfeagle inv 2/5/26</t>
+          <t>Shop price list 6/26/26</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Mops</t>
+          <t>Roller frames 9" HD</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Mop</t>
+          <t>C&amp;R 9" heavy duty roller frame #RF9HDN1</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Job</t>
+          <t>Bonding adhesive application</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>7.15</v>
+        <v>2.7</v>
       </c>
       <c r="G21" s="4">
         <f>D21*F21</f>
@@ -1171,40 +1171,114 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
+          <t>Gulfeagle inv 2/5/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Roller covers 9" 3/4" nap</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>C&amp;R 9" roller cover 3/4" nap #RC9-3/4</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Bonding adhesive application</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G22" s="4">
+        <f>D22*F22</f>
+        <v/>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Gulfeagle inv 2/5/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Mops</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Mop</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="G23" s="4">
+        <f>D23*F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
           <t>Shop price list 6/26/26</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>Material subtotal</t>
-        </is>
-      </c>
-      <c r="G23" s="6">
-        <f>SUM(G4:G21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Sales tax 7%</t>
-        </is>
-      </c>
-      <c r="G24" s="6">
-        <f>ROUND(G23*0.07,2)</f>
-        <v/>
       </c>
     </row>
     <row r="25">
       <c r="F25" s="5" t="inlineStr">
         <is>
+          <t>Material subtotal</t>
+        </is>
+      </c>
+      <c r="G25" s="6">
+        <f>SUM(G4:G23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Sales tax 7%</t>
+        </is>
+      </c>
+      <c r="G26" s="6">
+        <f>ROUND(G25*0.07,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="F27" s="5" t="inlineStr">
+        <is>
           <t>TOTAL MATERIAL</t>
         </is>
       </c>
-      <c r="G25" s="6">
-        <f>G23+G24</f>
+      <c r="G27" s="6">
+        <f>G25+G26</f>
         <v/>
       </c>
     </row>

</xml_diff>